<commit_message>
Deploying to gh-pages from @ jefersonrl/AgroSUS-FHIR@9d55176a67ba2317f47a61f6245676e13835474e 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-agrosus-atendimento-ubs.xlsx
+++ b/StructureDefinition-agrosus-atendimento-ubs.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-21T12:10:06+00:00</t>
+    <t>2026-07-21T12:21:04+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1323,7 +1323,7 @@
     <t>Categoria ou tipo de local após a alta</t>
   </si>
   <si>
-    <t>https://terminologia.saude.gov.br/fhir/CodeSystem/BRMotivoDesfecho</t>
+    <t>https://terminologia.saude.gov.br/fhir/ValueSet/BRMotivoDesfecho</t>
   </si>
   <si>
     <t>.dischargeDispositionCode</t>

</xml_diff>